<commit_message>
Fixes the production version
The production version works now íf the correct information is used
</commit_message>
<xml_diff>
--- a/data/busdata.xlsx
+++ b/data/busdata.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="39">
   <si>
     <t>Linje</t>
   </si>
@@ -40,10 +40,10 @@
     <t>Tillgängliga Lägen</t>
   </si>
   <si>
-    <t>Uppsala Lundellska skolan</t>
+    <t>Uppsala Lägerhyddsvägen</t>
   </si>
   <si>
-    <t>C</t>
+    <t>A</t>
   </si>
   <si>
     <t>Boländerna Gränbystaden</t>
@@ -55,10 +55,10 @@
     <t>Akademiska sjukhuset Ekonomikum</t>
   </si>
   <si>
-    <t>A</t>
+    <t>Uppsala Lundellska skolan</t>
   </si>
   <si>
-    <t>D</t>
+    <t>B</t>
   </si>
   <si>
     <t>Rosendal Akademiska sjukhuset</t>
@@ -70,19 +70,22 @@
     <t>Uppsala Polacksbacken</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>Uppsala Regementsvägen</t>
   </si>
   <si>
     <t>Nyby</t>
   </si>
   <si>
-    <t>Östra Gottsunda</t>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Rosendal Östra Gottsunda</t>
   </si>
   <si>
     <t>Campus Ultuna</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
   <si>
     <t>Gränbystaden Norra Årsta</t>
@@ -91,7 +94,7 @@
     <t>Centralstationen</t>
   </si>
   <si>
-    <t>Ultuna Gottsunda</t>
+    <t>Ulleråker Ultuna Gottsunda</t>
   </si>
   <si>
     <t>Engelska skolan</t>
@@ -118,7 +121,13 @@
     <t>Ulleråker Ultuna</t>
   </si>
   <si>
+    <t>Ultuna Gottsunda</t>
+  </si>
+  <si>
     <t>Uppsala</t>
+  </si>
+  <si>
+    <t>Östra Gottsunda</t>
   </si>
 </sst>
 </file>
@@ -355,7 +364,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="G1:J1000" displayName="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="G1:J1000" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -652,10 +661,10 @@
         <v>13</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I2" s="14" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J2" s="14"/>
       <c r="K2" s="15"/>
@@ -697,7 +706,7 @@
         <v>18</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J3" s="17"/>
       <c r="K3" s="15"/>
@@ -722,13 +731,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -736,10 +745,10 @@
         <v>11</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="J4" s="17"/>
       <c r="K4" s="15"/>
@@ -764,10 +773,10 @@
         <v>3.0</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>22</v>
@@ -779,7 +788,7 @@
       </c>
       <c r="H5" s="19"/>
       <c r="I5" s="11" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="J5" s="17"/>
       <c r="K5" s="15"/>
@@ -807,15 +816,15 @@
         <v>18</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
       <c r="G6" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="19"/>
       <c r="I6" s="19"/>
@@ -845,15 +854,15 @@
         <v>18</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E7" s="15"/>
       <c r="F7" s="15"/>
       <c r="G7" s="11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H7" s="19"/>
       <c r="I7" s="19"/>
@@ -880,17 +889,17 @@
         <v>8.0</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H8" s="19"/>
       <c r="I8" s="19"/>
@@ -917,17 +926,17 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F9" s="15"/>
       <c r="G9" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H9" s="19"/>
       <c r="I9" s="19"/>
@@ -954,17 +963,17 @@
         <v>11.0</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H10" s="19"/>
       <c r="I10" s="19"/>
@@ -991,18 +1000,18 @@
         <v>11.0</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E11" s="15"/>
       <c r="F11" s="15"/>
       <c r="G11" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H11" s="19"/>
       <c r="I11" s="19"/>
@@ -1032,10 +1041,10 @@
         <v>18</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F12" s="15"/>
       <c r="G12" s="11" t="s">
@@ -1069,15 +1078,15 @@
         <v>18</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
       <c r="G13" s="12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H13" s="19"/>
       <c r="I13" s="19"/>
@@ -1107,7 +1116,7 @@
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
       <c r="G14" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H14" s="19"/>
       <c r="I14" s="19"/>
@@ -1137,7 +1146,7 @@
       <c r="E15" s="15"/>
       <c r="F15" s="15"/>
       <c r="G15" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H15" s="19"/>
       <c r="I15" s="19"/>
@@ -1166,7 +1175,7 @@
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
       <c r="G16" s="11" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="H16" s="19"/>
       <c r="I16" s="19"/>
@@ -1195,7 +1204,7 @@
       <c r="E17" s="15"/>
       <c r="F17" s="15"/>
       <c r="G17" s="11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H17" s="19"/>
       <c r="I17" s="19"/>
@@ -1224,7 +1233,7 @@
       <c r="E18" s="15"/>
       <c r="F18" s="15"/>
       <c r="G18" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H18" s="19"/>
       <c r="I18" s="19"/>
@@ -1253,7 +1262,7 @@
       <c r="E19" s="15"/>
       <c r="F19" s="15"/>
       <c r="G19" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H19" s="19"/>
       <c r="I19" s="19"/>
@@ -1283,7 +1292,7 @@
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
       <c r="G20" s="11" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="H20" s="19"/>
       <c r="I20" s="19"/>

</xml_diff>